<commit_message>
Store each Bale user in Cloudflare D1.
Upsert the sender on every message or callback, and let the admin list recent users with /users. Document how to create the database, bind it, and migrate a Worker that is already deployed.

Add Persian comments that explain the existing bot modules. Regenerate sample.xlsx so its zip checksum is valid.

Co-authored-by: arghavanreza <arghavanreza@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/sample.xlsx
+++ b/assets/sample.xlsx
@@ -13,6 +13,116 @@
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Add transfer menus, channel checks, and paya ccti files.
Customers can request a sample workbook, confirm a single transfer, or upload a group list. Each row is classified as internal, paya, or satna, and only paya rows become a Bank Mehr .ccti file for the admin.

Co-authored-by: arghavanreza <arghavanreza@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/sample.xlsx
+++ b/assets/sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="payments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="transfers" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ignore-me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -414,23 +414,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>نام ذینفع</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>کدملی</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>sheba</t>
+          <t>شماره شبا / حساب ذینفع</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>مبلغ</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>شناسه واریز</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>شرح</t>
         </is>
       </c>
     </row>
@@ -440,12 +455,27 @@
           <t>علی رضایی</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0084575948</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>IR300600000000000000000001</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>1500000</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>IR430120000000000000000001</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>حقوق</t>
         </is>
       </c>
     </row>
@@ -455,12 +485,52 @@
           <t>سارا محمدی</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>IR160120000000000000000002</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>250000</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>IR490170000000000000000002</t>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>رضا کریمی</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>IR220170000000000000000003</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>نمونه ساتنا</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>نرگس احمدی</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1234567890123</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>حساب مهر</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add customer transfer menus and paya ccti files
Customers can request a sample workbook, confirm a single transfer, or upload a group list. Each row is classified as internal, paya, or satna, and only paya rows become a Bank Mehr .ccti file for the admin.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: arghavanreza <arghavanreza@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/sample.xlsx
+++ b/assets/sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="payments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="transfers" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ignore-me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -414,23 +414,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>نام ذینفع</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>کدملی</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>sheba</t>
+          <t>شماره شبا / حساب ذینفع</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>مبلغ</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>شناسه واریز</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>شرح</t>
         </is>
       </c>
     </row>
@@ -440,12 +455,27 @@
           <t>علی رضایی</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0084575948</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>IR300600000000000000000001</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>1500000</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>IR430120000000000000000001</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>حقوق</t>
         </is>
       </c>
     </row>
@@ -455,12 +485,52 @@
           <t>سارا محمدی</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>IR160120000000000000000002</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>250000</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>IR490170000000000000000002</t>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>رضا کریمی</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>IR220170000000000000000003</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>نمونه ساتنا</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>نرگس احمدی</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1234567890123</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>حساب مهر</t>
         </is>
       </c>
     </row>

</xml_diff>